<commit_message>
Cost calculator and profile
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/03_Profile/Profile/01_ProfileTest.xlsx
+++ b/src/test/resources/testdata/Modules/03_Profile/Profile/01_ProfileTest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\03_Profile\Profile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549CE78E-205A-4F78-9A8D-29B4B3071148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFE9D6B-6964-43B5-A220-C9AA412F3814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1610" windowWidth="19200" windowHeight="9190" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="94">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -246,21 +246,12 @@
     <t>ProfileTest_20</t>
   </si>
   <si>
-    <t>Verify horizontal scroll for milestones</t>
-  </si>
-  <si>
-    <t>verifymilestonehorizontalscroll</t>
-  </si>
-  <si>
     <t>Verify influencer image</t>
   </si>
   <si>
     <t>verifyinfluencerimageondisplay</t>
   </si>
   <si>
-    <t>0.000</t>
-  </si>
-  <si>
     <t>admin@gmail.com</t>
   </si>
   <si>
@@ -282,9 +273,6 @@
     <t>English</t>
   </si>
   <si>
-    <t>Version : 1.304.54-Test</t>
-  </si>
-  <si>
     <t>Last status changed on -</t>
   </si>
   <si>
@@ -294,102 +282,24 @@
     <t>ProfileTest_22</t>
   </si>
   <si>
-    <t>clickonsignout veriftysignoutlable</t>
-  </si>
-  <si>
     <t>Verify Signout lable</t>
   </si>
   <si>
     <t>Logout</t>
   </si>
   <si>
-    <t>ProfileTest_23</t>
-  </si>
-  <si>
     <t>Click On signout-NO</t>
   </si>
   <si>
     <t>clickonnosignout</t>
   </si>
   <si>
-    <t>clickondeleteaccountbtn verifydeleteaccounttitle</t>
-  </si>
-  <si>
-    <t>verifydeleteaccountmsg</t>
-  </si>
-  <si>
-    <t>clickonsubmitbtndeleteacc verifydeleteaccerrormsg</t>
-  </si>
-  <si>
-    <t>verifydeleteaccinfname</t>
-  </si>
-  <si>
-    <t>clickondeleteaccnobtn</t>
-  </si>
-  <si>
-    <t>2602000006</t>
-  </si>
-  <si>
-    <t>2602000007</t>
-  </si>
-  <si>
-    <t>2602000008</t>
-  </si>
-  <si>
-    <t>2602000009</t>
-  </si>
-  <si>
-    <t>2602000010</t>
-  </si>
-  <si>
-    <t>ProfileTest_24</t>
-  </si>
-  <si>
-    <t>ProfileTest_25</t>
-  </si>
-  <si>
-    <t>ProfileTest_26</t>
-  </si>
-  <si>
-    <t>ProfileTest_27</t>
-  </si>
-  <si>
-    <t>ProfileTest_28</t>
-  </si>
-  <si>
-    <t>Verify delete account dialog title</t>
-  </si>
-  <si>
-    <t>Verify delete account dialog msg</t>
-  </si>
-  <si>
-    <t>verify delete account error msg</t>
-  </si>
-  <si>
-    <t>verify delete account inf name</t>
-  </si>
-  <si>
-    <t>close delete account dialog</t>
-  </si>
-  <si>
-    <t>Delete My Account</t>
-  </si>
-  <si>
-    <t>You have requested to delete your account. We will immediately submit the request to delete your account.  Our system will delete all your data other than the data which needs to be retained as per various taxation, data retention policies specified by Government of India being the regulatory requirements.</t>
-  </si>
-  <si>
-    <t>Captcha is invalid.</t>
-  </si>
-  <si>
     <t>03_PROFILE</t>
   </si>
   <si>
     <t>Appium Auto_Influencer_002  | Electrical Contractor | Base</t>
   </si>
   <si>
-    <t>0.00</t>
-  </si>
-  <si>
     <t>Automation  Firm</t>
   </si>
   <si>
@@ -397,13 +307,23 @@
   </si>
   <si>
     <t>14,  Kai Nanasaheb Sutar Path,  Gujrat Colony,  Kothrud, Pune, Pune City,  Pune,  Maharashtra 411038,  India</t>
+  </si>
+  <si>
+    <t>-Test</t>
+  </si>
+  <si>
+    <t>CONTAINS</t>
+  </si>
+  <si>
+    <t>clickonsignout
+veriftysignoutlable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -558,8 +478,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -742,6 +669,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -947,7 +880,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -961,10 +894,14 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="10" xfId="43" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="21" fillId="34" borderId="10" xfId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1342,7 +1279,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{089D5808-B2AF-4105-BEF8-05FAA4CBE122}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1383,7 +1320,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>10</v>
@@ -1406,7 +1343,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>11</v>
@@ -1418,7 +1355,7 @@
         <v>30</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -1429,7 +1366,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -1440,8 +1377,8 @@
       <c r="E4" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>76</v>
+      <c r="F4" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>5</v>
@@ -1452,7 +1389,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>13</v>
@@ -1463,8 +1400,8 @@
       <c r="E5" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>77</v>
+      <c r="F5" s="11" t="s">
+        <v>74</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>5</v>
@@ -1475,7 +1412,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
@@ -1486,7 +1423,7 @@
       <c r="E6" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="11" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -1498,7 +1435,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>15</v>
@@ -1509,8 +1446,8 @@
       <c r="E7" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>75</v>
+      <c r="F7" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>5</v>
@@ -1521,7 +1458,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>16</v>
@@ -1532,7 +1469,7 @@
       <c r="E8" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="11" t="s">
         <v>40</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -1544,7 +1481,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>17</v>
@@ -1556,7 +1493,7 @@
         <v>44</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>5</v>
@@ -1567,7 +1504,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
@@ -1579,7 +1516,7 @@
         <v>45</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>5</v>
@@ -1590,7 +1527,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>19</v>
@@ -1602,7 +1539,7 @@
         <v>46</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>117</v>
+        <v>8</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>5</v>
@@ -1613,7 +1550,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>20</v>
@@ -1624,8 +1561,8 @@
       <c r="E12" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>118</v>
+      <c r="F12" s="9" t="s">
+        <v>88</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>5</v>
@@ -1636,7 +1573,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
@@ -1648,7 +1585,7 @@
         <v>50</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>5</v>
@@ -1659,7 +1596,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>22</v>
@@ -1671,7 +1608,7 @@
         <v>52</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>5</v>
@@ -1682,7 +1619,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>23</v>
@@ -1693,8 +1630,8 @@
       <c r="E15" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>78</v>
+      <c r="F15" s="11" t="s">
+        <v>75</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>5</v>
@@ -1705,7 +1642,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>24</v>
@@ -1716,8 +1653,8 @@
       <c r="E16" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>79</v>
+      <c r="F16" s="11" t="s">
+        <v>76</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>5</v>
@@ -1728,7 +1665,7 @@
         <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>25</v>
@@ -1739,8 +1676,8 @@
       <c r="E17" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>80</v>
+      <c r="F17" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>5</v>
@@ -1751,7 +1688,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>26</v>
@@ -1762,8 +1699,8 @@
       <c r="E18" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>81</v>
+      <c r="F18" s="11" t="s">
+        <v>78</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>5</v>
@@ -1774,7 +1711,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>67</v>
@@ -1786,7 +1723,7 @@
         <v>62</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>5</v>
@@ -1797,7 +1734,7 @@
         <v>9</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>68</v>
@@ -1809,10 +1746,10 @@
         <v>64</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>5</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -1820,7 +1757,7 @@
         <v>9</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>69</v>
@@ -1838,24 +1775,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>73</v>
+        <v>82</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>93</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>8</v>
+        <v>83</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>5</v>
@@ -1866,159 +1803,21 @@
         <v>9</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>86</v>
-      </c>
       <c r="F23" s="1" t="s">
-        <v>88</v>
+        <v>8</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="92.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G29" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Claim Points & Profile failed Testcases updated.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/03_Profile/Profile/01_ProfileTest.xlsx
+++ b/src/test/resources/testdata/Modules/03_Profile/Profile/01_ProfileTest.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\03_Profile\Profile\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\03_Profile\Profile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFE9D6B-6964-43B5-A220-C9AA412F3814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574BFF9C-1C49-4BE7-A12C-15ADDE708D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="91">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -246,12 +246,6 @@
     <t>ProfileTest_20</t>
   </si>
   <si>
-    <t>Verify influencer image</t>
-  </si>
-  <si>
-    <t>verifyinfluencerimageondisplay</t>
-  </si>
-  <si>
     <t>admin@gmail.com</t>
   </si>
   <si>
@@ -277,9 +271,6 @@
   </si>
   <si>
     <t>ProfileTest_21</t>
-  </si>
-  <si>
-    <t>ProfileTest_22</t>
   </si>
   <si>
     <t>Verify Signout lable</t>
@@ -1279,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{089D5808-B2AF-4105-BEF8-05FAA4CBE122}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1320,7 +1311,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>10</v>
@@ -1343,7 +1334,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>11</v>
@@ -1355,7 +1346,7 @@
         <v>30</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -1366,7 +1357,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -1378,7 +1369,7 @@
         <v>66</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>5</v>
@@ -1389,7 +1380,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>13</v>
@@ -1401,7 +1392,7 @@
         <v>31</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>5</v>
@@ -1412,7 +1403,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
@@ -1435,7 +1426,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>15</v>
@@ -1447,7 +1438,7 @@
         <v>37</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>5</v>
@@ -1458,7 +1449,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>16</v>
@@ -1481,7 +1472,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>17</v>
@@ -1504,7 +1495,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
@@ -1527,7 +1518,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>19</v>
@@ -1550,7 +1541,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>20</v>
@@ -1562,7 +1553,7 @@
         <v>48</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>5</v>
@@ -1573,7 +1564,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
@@ -1585,7 +1576,7 @@
         <v>50</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>5</v>
@@ -1596,7 +1587,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>22</v>
@@ -1608,7 +1599,7 @@
         <v>52</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>5</v>
@@ -1619,7 +1610,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>23</v>
@@ -1631,7 +1622,7 @@
         <v>54</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>5</v>
@@ -1642,7 +1633,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>24</v>
@@ -1654,7 +1645,7 @@
         <v>56</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>5</v>
@@ -1665,7 +1656,7 @@
         <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>25</v>
@@ -1677,7 +1668,7 @@
         <v>58</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>5</v>
@@ -1688,7 +1679,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>26</v>
@@ -1700,7 +1691,7 @@
         <v>60</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>5</v>
@@ -1711,7 +1702,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>67</v>
@@ -1723,7 +1714,7 @@
         <v>62</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>5</v>
@@ -1734,7 +1725,7 @@
         <v>9</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>68</v>
@@ -1746,78 +1737,55 @@
         <v>64</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>69</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>71</v>
+        <v>79</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="F21" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="G22" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G23" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Resolved Failed TestCases - 14-04-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/03_Profile/Profile/01_ProfileTest.xlsx
+++ b/src/test/resources/testdata/Modules/03_Profile/Profile/01_ProfileTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\03_Profile\Profile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574BFF9C-1C49-4BE7-A12C-15ADDE708D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEE2B7D5-A3E4-43CA-8DC7-0A32335059C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -282,9 +282,6 @@
     <t>Click On signout-NO</t>
   </si>
   <si>
-    <t>clickonnosignout</t>
-  </si>
-  <si>
     <t>03_PROFILE</t>
   </si>
   <si>
@@ -308,6 +305,10 @@
   <si>
     <t>clickonsignout
 veriftysignoutlable</t>
+  </si>
+  <si>
+    <t>clickonnosignout
+navigatebacktodashboardpage</t>
   </si>
 </sst>
 </file>
@@ -1311,7 +1312,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>10</v>
@@ -1334,7 +1335,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>11</v>
@@ -1346,7 +1347,7 @@
         <v>30</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>5</v>
@@ -1357,7 +1358,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -1380,7 +1381,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>13</v>
@@ -1403,7 +1404,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
@@ -1426,7 +1427,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>15</v>
@@ -1449,7 +1450,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>16</v>
@@ -1472,7 +1473,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>17</v>
@@ -1495,7 +1496,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
@@ -1518,7 +1519,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>19</v>
@@ -1541,7 +1542,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>20</v>
@@ -1553,7 +1554,7 @@
         <v>48</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>5</v>
@@ -1564,7 +1565,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
@@ -1576,7 +1577,7 @@
         <v>50</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>5</v>
@@ -1587,7 +1588,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>22</v>
@@ -1599,7 +1600,7 @@
         <v>52</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>5</v>
@@ -1610,7 +1611,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>23</v>
@@ -1633,7 +1634,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>24</v>
@@ -1656,7 +1657,7 @@
         <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>25</v>
@@ -1679,7 +1680,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>26</v>
@@ -1702,7 +1703,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>67</v>
@@ -1725,7 +1726,7 @@
         <v>9</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>68</v>
@@ -1737,10 +1738,10 @@
         <v>64</v>
       </c>
       <c r="F20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -1748,7 +1749,7 @@
         <v>9</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>69</v>
@@ -1757,7 +1758,7 @@
         <v>79</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>80</v>
@@ -1766,12 +1767,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>78</v>
@@ -1779,8 +1780,8 @@
       <c r="D22" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>82</v>
+      <c r="E22" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>8</v>

</xml_diff>